<commit_message>
update: add login test cases and split API login into success and failure
</commit_message>
<xml_diff>
--- a/00.test_case/Demoblaze_TestCases_Login_Cart.xlsx
+++ b/00.test_case/Demoblaze_TestCases_Login_Cart.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
   <si>
     <t xml:space="preserve">Demoblaze – Test Case Suite (Login, Cart &amp; Order)</t>
   </si>
@@ -508,7 +508,7 @@
     <t xml:space="preserve">Input treated as empty: validation alert shown, no login request is accepted; user not logged in</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm trimming rule with BA</t>
+    <t xml:space="preserve">Alert 'Wrong password.' shown; whitespace input is sent to the API and an account with a whitespace-only username exists</t>
   </si>
   <si>
     <t>LG-017</t>
@@ -568,6 +568,9 @@
     <t xml:space="preserve">System applies one consistent rule: either input is trimmed and login succeeds, or login fails with an error alert. No partial/broken session</t>
   </si>
   <si>
+    <t xml:space="preserve">Confirm trimming rule with BA</t>
+  </si>
+  <si>
     <t>LG-020</t>
   </si>
   <si>
@@ -592,7 +595,7 @@
     <t>LG-021</t>
   </si>
   <si>
-    <t xml:space="preserve">Very long username (300 characters)</t>
+    <t xml:space="preserve">Very long username (2000 characters)</t>
   </si>
   <si>
     <t xml:space="preserve">Username: 'a' x 300
@@ -605,6 +608,9 @@
   </si>
   <si>
     <t xml:space="preserve">Error alert shown; page remains responsive; no server error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No alert is shown, the Log in modal stays open and the user gets no feedback.</t>
   </si>
   <si>
     <t>LG-022</t>
@@ -1274,7 +1280,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -1305,6 +1311,11 @@
       <b/>
       <sz val="11.000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9.000000"/>
+      <color rgb="FF8C8C8C"/>
+      <name val="Courier New"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1371,7 +1382,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" quotePrefix="0" pivotButton="0"/>
@@ -1406,6 +1417,9 @@
     </xf>
     <xf fontId="1" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2085,11 +2099,11 @@
       </c>
       <c r="B18" s="7">
         <f>COUNTIF(Login!$M:$M,"Pass")</f>
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="C18" s="7">
         <f>COUNTIF(Login!$M:$M,"Fail")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" s="7">
         <f>COUNTIF(Login!$M:$M,"Blocked")</f>
@@ -2097,11 +2111,11 @@
       </c>
       <c r="E18" s="7">
         <f>COUNTIF(Login!$M:$M,"Not Run")</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F18" s="11">
         <f t="shared" ref="F18:F20" si="1">IFERROR(B18/(B18+C18+D18),0)</f>
-        <v>1</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -2204,7 +2218,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="10"/>
     <col customWidth="1" min="2" max="2" style="1" width="9"/>
@@ -2435,7 +2449,7 @@
         <v>72</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N5" s="13"/>
       <c r="O5" s="13"/>
@@ -2478,7 +2492,7 @@
         <v>72</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N6" s="13"/>
       <c r="O6" s="13"/>
@@ -2521,7 +2535,7 @@
         <v>56</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N7" s="13"/>
       <c r="O7" s="13"/>
@@ -2564,7 +2578,7 @@
         <v>56</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N8" s="13"/>
       <c r="O8" s="13"/>
@@ -2607,7 +2621,7 @@
         <v>65</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N9" s="13"/>
       <c r="O9" s="13" t="s">
@@ -2652,7 +2666,7 @@
         <v>106</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N10" s="13"/>
       <c r="O10" s="13" t="s">
@@ -2697,7 +2711,7 @@
         <v>114</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N11" s="13"/>
       <c r="O11" s="13"/>
@@ -2740,7 +2754,7 @@
         <v>114</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N12" s="13"/>
       <c r="O12" s="13"/>
@@ -2783,7 +2797,7 @@
         <v>114</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N13" s="13"/>
       <c r="O13" s="13"/>
@@ -2826,7 +2840,7 @@
         <v>129</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N14" s="13"/>
       <c r="O14" s="13"/>
@@ -2869,7 +2883,7 @@
         <v>129</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
@@ -2912,7 +2926,7 @@
         <v>65</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N16" s="13"/>
       <c r="O16" s="13"/>
@@ -2954,13 +2968,13 @@
       <c r="L17" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="M17" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13" t="s">
+      <c r="M17" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" s="13" t="s">
         <v>144</v>
       </c>
+      <c r="O17" s="13"/>
     </row>
     <row r="18" ht="35.049999999999997" customHeight="1">
       <c r="A18" s="13" t="s">
@@ -3000,7 +3014,7 @@
         <v>106</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N18" s="13"/>
       <c r="O18" s="13"/>
@@ -3043,7 +3057,7 @@
         <v>106</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N19" s="13"/>
       <c r="O19" s="13"/>
@@ -3086,16 +3100,16 @@
         <v>65</v>
       </c>
       <c r="M20" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N20" s="13"/>
       <c r="O20" s="13" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" ht="46.25" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>17</v>
@@ -3104,7 +3118,7 @@
         <v>58</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>14</v>
@@ -3116,13 +3130,13 @@
         <v>61</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K21" s="13" t="s">
         <v>55</v>
@@ -3131,16 +3145,16 @@
         <v>65</v>
       </c>
       <c r="M21" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N21" s="13"/>
       <c r="O21" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" ht="35.049999999999997" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B22" s="13" t="s">
         <v>17</v>
@@ -3149,7 +3163,7 @@
         <v>109</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>14</v>
@@ -3161,13 +3175,13 @@
         <v>51</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>55</v>
@@ -3175,15 +3189,17 @@
       <c r="L22" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="M22" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="N22" s="13"/>
+      <c r="M22" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N22" s="13" t="s">
+        <v>173</v>
+      </c>
       <c r="O22" s="13"/>
     </row>
     <row r="23" ht="46.25" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>17</v>
@@ -3192,7 +3208,7 @@
         <v>58</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>14</v>
@@ -3207,10 +3223,10 @@
         <v>103</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="K23" s="13" t="s">
         <v>55</v>
@@ -3219,14 +3235,14 @@
         <v>65</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N23" s="13"/>
       <c r="O23" s="13"/>
     </row>
     <row r="24" ht="23.850000000000001" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B24" s="13" t="s">
         <v>17</v>
@@ -3235,7 +3251,7 @@
         <v>67</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>14</v>
@@ -3244,16 +3260,16 @@
         <v>75</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H24" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K24" s="13" t="s">
         <v>55</v>
@@ -3262,14 +3278,14 @@
         <v>72</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
     </row>
     <row r="25" ht="46.25" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>17</v>
@@ -3278,7 +3294,7 @@
         <v>67</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>12</v>
@@ -3293,10 +3309,10 @@
         <v>103</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J25" s="13" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K25" s="13" t="s">
         <v>55</v>
@@ -3305,23 +3321,23 @@
         <v>72</v>
       </c>
       <c r="M25" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N25" s="13"/>
       <c r="O25" s="13"/>
     </row>
     <row r="26" ht="23.850000000000001" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B26" s="13" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>12</v>
@@ -3330,25 +3346,25 @@
         <v>60</v>
       </c>
       <c r="G26" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="K26" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="H26" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="J26" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="K26" s="13" t="s">
-        <v>186</v>
-      </c>
       <c r="L26" s="13" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="M26" s="13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
@@ -3404,18 +3420,1644 @@
           </x14:cfRule>
           <xm:sqref>M2:M26</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{7A055AB6-F9B4-4D89-A286-8236C0E60A0A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9" disablePrompts="0">
+        <x14:dataValidation xr:uid="{1C1F83F4-DCAD-4900-9F08-46A0ED2A5702}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>M2:M26</xm:sqref>
+          <xm:sqref>M2:M16</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{29D6183F-1C3D-484B-A87B-EBF39946C35D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{701A93A6-75E2-45E9-8984-1EB581FEC577}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M19</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{412503E6-BDBA-4824-ACE6-C26B86AF95DE}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M20</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{3509C0B1-35D4-471B-A8FD-4F06F0E94DB4}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M21</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{54381B46-38F3-4496-A12F-77B4E4F9B3AA}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M23</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{2FF03370-1799-4664-8B94-7F26FF05D694}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M24</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{15F726E3-4587-4069-8DFF-84B80575A152}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M25</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{05AD8129-44E8-4D45-B5BF-17BD74FCB627}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>M26</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3495,16 +5137,16 @@
     </row>
     <row r="2" ht="46.25" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>12</v>
@@ -3516,19 +5158,19 @@
         <v>51</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="K2" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L2" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M2" s="13" t="s">
         <v>24</v>
@@ -3538,16 +5180,16 @@
     </row>
     <row r="3" ht="46.25" customHeight="1">
       <c r="A3" s="13" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>12</v>
@@ -3556,22 +5198,22 @@
         <v>60</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="K3" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L3" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M3" s="13" t="s">
         <v>24</v>
@@ -3581,16 +5223,16 @@
     </row>
     <row r="4" ht="35.049999999999997" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>12</v>
@@ -3602,19 +5244,19 @@
         <v>51</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="K4" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L4" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M4" s="13" t="s">
         <v>24</v>
@@ -3624,16 +5266,16 @@
     </row>
     <row r="5" ht="35.049999999999997" customHeight="1">
       <c r="A5" s="13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>14</v>
@@ -3645,40 +5287,40 @@
         <v>51</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="K5" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>24</v>
       </c>
       <c r="N5" s="13"/>
       <c r="O5" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" ht="23.850000000000001" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>12</v>
@@ -3687,22 +5329,22 @@
         <v>60</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="K6" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M6" s="13" t="s">
         <v>24</v>
@@ -3712,16 +5354,16 @@
     </row>
     <row r="7" ht="23.850000000000001" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>12</v>
@@ -3730,22 +5372,22 @@
         <v>50</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M7" s="13" t="s">
         <v>24</v>
@@ -3755,16 +5397,16 @@
     </row>
     <row r="8" ht="23.850000000000001" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>12</v>
@@ -3773,22 +5415,22 @@
         <v>50</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H8" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="M8" s="13" t="s">
         <v>24</v>
@@ -3798,16 +5440,16 @@
     </row>
     <row r="9" ht="57.450000000000003" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>12</v>
@@ -3816,22 +5458,22 @@
         <v>50</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="K9" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="M9" s="13" t="s">
         <v>24</v>
@@ -3841,16 +5483,16 @@
     </row>
     <row r="10" ht="35.049999999999997" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>12</v>
@@ -3859,22 +5501,22 @@
         <v>86</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L10" s="13" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="M10" s="13" t="s">
         <v>24</v>
@@ -3884,16 +5526,16 @@
     </row>
     <row r="11" ht="35.049999999999997" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>12</v>
@@ -3905,19 +5547,19 @@
         <v>51</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="K11" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L11" s="13" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="M11" s="13" t="s">
         <v>24</v>
@@ -3927,16 +5569,16 @@
     </row>
     <row r="12" ht="35.049999999999997" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>12</v>
@@ -3948,19 +5590,19 @@
         <v>51</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="K12" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L12" s="13" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="M12" s="13" t="s">
         <v>24</v>
@@ -3970,16 +5612,16 @@
     </row>
     <row r="13" ht="23.850000000000001" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E13" s="16" t="s">
         <v>13</v>
@@ -3988,22 +5630,22 @@
         <v>50</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="K13" s="13" t="s">
         <v>128</v>
       </c>
       <c r="L13" s="13" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="M13" s="13" t="s">
         <v>24</v>
@@ -4013,16 +5655,16 @@
     </row>
     <row r="14" ht="23.850000000000001" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E14" s="16" t="s">
         <v>13</v>
@@ -4031,22 +5673,22 @@
         <v>60</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L14" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="M14" s="13" t="s">
         <v>24</v>
@@ -4056,16 +5698,16 @@
     </row>
     <row r="15" ht="23.850000000000001" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E15" s="16" t="s">
         <v>13</v>
@@ -4074,22 +5716,22 @@
         <v>75</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L15" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="M15" s="13" t="s">
         <v>24</v>
@@ -4099,16 +5741,16 @@
     </row>
     <row r="16" ht="35.049999999999997" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>14</v>
@@ -4120,40 +5762,40 @@
         <v>51</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="K16" s="13" t="s">
         <v>128</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M16" s="13" t="s">
         <v>24</v>
       </c>
       <c r="N16" s="13"/>
       <c r="O16" s="13" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="17" ht="23.850000000000001" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>14</v>
@@ -4162,22 +5804,22 @@
         <v>75</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L17" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M17" s="13" t="s">
         <v>24</v>
@@ -4187,16 +5829,16 @@
     </row>
     <row r="18" ht="35.049999999999997" customHeight="1">
       <c r="A18" s="13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>14</v>
@@ -4208,19 +5850,19 @@
         <v>51</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="K18" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L18" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M18" s="13" t="s">
         <v>24</v>
@@ -4230,16 +5872,16 @@
     </row>
     <row r="19" ht="46.25" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>12</v>
@@ -4248,22 +5890,22 @@
         <v>50</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L19" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="M19" s="13" t="s">
         <v>24</v>
@@ -4340,7 +5982,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{51D5044C-EC53-49BD-8854-157F2F9BE87A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{49C9940B-44B3-475D-B2CB-BD180AEDD24E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -4424,16 +6066,16 @@
     </row>
     <row r="2" ht="23.850000000000001" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>12</v>
@@ -4442,22 +6084,22 @@
         <v>50</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H2" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="K2" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L2" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M2" s="13" t="s">
         <v>24</v>
@@ -4467,16 +6109,16 @@
     </row>
     <row r="3" ht="68.650000000000006" customHeight="1">
       <c r="A3" s="13" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>12</v>
@@ -4485,22 +6127,22 @@
         <v>60</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="K3" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L3" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M3" s="13" t="s">
         <v>24</v>
@@ -4510,16 +6152,16 @@
     </row>
     <row r="4" ht="35.049999999999997" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>12</v>
@@ -4528,22 +6170,22 @@
         <v>50</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K4" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L4" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M4" s="13" t="s">
         <v>24</v>
@@ -4553,16 +6195,16 @@
     </row>
     <row r="5" ht="35.049999999999997" customHeight="1">
       <c r="A5" s="13" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>12</v>
@@ -4571,22 +6213,22 @@
         <v>60</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="K5" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>24</v>
@@ -4596,16 +6238,16 @@
     </row>
     <row r="6" ht="23.850000000000001" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>13</v>
@@ -4614,22 +6256,22 @@
         <v>50</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="K6" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M6" s="13" t="s">
         <v>24</v>
@@ -4639,16 +6281,16 @@
     </row>
     <row r="7" ht="35.049999999999997" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E7" s="16" t="s">
         <v>13</v>
@@ -4657,22 +6299,22 @@
         <v>50</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M7" s="13" t="s">
         <v>24</v>
@@ -4682,16 +6324,16 @@
     </row>
     <row r="8" ht="35.049999999999997" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E8" s="16" t="s">
         <v>13</v>
@@ -4700,22 +6342,22 @@
         <v>50</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M8" s="13" t="s">
         <v>24</v>
@@ -4725,16 +6367,16 @@
     </row>
     <row r="9" ht="46.25" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E9" s="16" t="s">
         <v>13</v>
@@ -4743,22 +6385,22 @@
         <v>75</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="K9" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M9" s="13" t="s">
         <v>24</v>
@@ -4768,16 +6410,16 @@
     </row>
     <row r="10" ht="35.049999999999997" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>13</v>
@@ -4786,43 +6428,43 @@
         <v>50</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L10" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M10" s="13" t="s">
         <v>24</v>
       </c>
       <c r="N10" s="13"/>
       <c r="O10" s="13" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" ht="35.049999999999997" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>13</v>
@@ -4831,43 +6473,43 @@
         <v>75</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="K11" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L11" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M11" s="13" t="s">
         <v>24</v>
       </c>
       <c r="N11" s="13"/>
       <c r="O11" s="13" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" ht="35.049999999999997" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>13</v>
@@ -4876,43 +6518,43 @@
         <v>50</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="K12" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L12" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M12" s="13" t="s">
         <v>24</v>
       </c>
       <c r="N12" s="13"/>
       <c r="O12" s="13" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" ht="23.850000000000001" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>14</v>
@@ -4921,22 +6563,22 @@
         <v>75</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="K13" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L13" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M13" s="13" t="s">
         <v>24</v>
@@ -4946,16 +6588,16 @@
     </row>
     <row r="14" ht="23.850000000000001" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>14</v>
@@ -4964,22 +6606,22 @@
         <v>86</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="K14" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L14" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M14" s="13" t="s">
         <v>24</v>
@@ -4989,16 +6631,16 @@
     </row>
     <row r="15" ht="35.049999999999997" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>14</v>
@@ -5007,22 +6649,22 @@
         <v>86</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="K15" s="13" t="s">
         <v>55</v>
       </c>
       <c r="L15" s="13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M15" s="13" t="s">
         <v>24</v>
@@ -5103,7 +6745,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{40237662-67AD-4676-8847-52828C683044}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{05693C4F-E1C2-472E-B7C5-440663D94E2D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>

</xml_diff>

<commit_message>
update: update test script cart
</commit_message>
<xml_diff>
--- a/00.test_case/Demoblaze_TestCases_Login_Cart.xlsx
+++ b/00.test_case/Demoblaze_TestCases_Login_Cart.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -947,7 +947,7 @@
     <t>CT-015</t>
   </si>
   <si>
-    <t xml:space="preserve">Add many items (10)</t>
+    <t xml:space="preserve">Add many items (10) or max</t>
   </si>
   <si>
     <t xml:space="preserve">10 x add to cart via API</t>
@@ -957,7 +957,7 @@
 2. Open 'Cart'</t>
   </si>
   <si>
-    <t xml:space="preserve">10 rows listed; total equals sum of prices</t>
+    <t xml:space="preserve">10 (max) rows listed; total equals sum of prices</t>
   </si>
   <si>
     <t xml:space="preserve">Items seeded via API to speed up setup</t>
@@ -2108,7 +2108,7 @@
         <v>0.92</v>
       </c>
       <c r="G18" s="12">
-        <f>1-E18/E11</f>
+        <f t="shared" ref="G18:G20" si="2">1-E18/E11</f>
         <v>1</v>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="B19" s="7">
         <f>COUNTIF(Cart!$M:$M,"Pass")</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C19" s="7">
         <f>COUNTIF(Cart!$M:$M,"Fail")</f>
@@ -2130,15 +2130,15 @@
       </c>
       <c r="E19" s="7">
         <f>COUNTIF(Cart!$M:$M,"Not Run")</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="12">
-        <f>1-E19/E12</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -2166,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="12">
-        <f>1-E20/E13</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5017,7 +5017,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9" disablePrompts="0">
-        <x14:dataValidation xr:uid="{6ADE8671-DDC5-4207-A0BA-BA3AC60B27C8}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{7D526BDB-C970-4102-88CF-19C2D028DEC3}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5026,7 +5026,7 @@
           </x14:formula2>
           <xm:sqref>M2:M16</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{5476ACE9-6595-41E2-959D-B7ECEBE1FAE0}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{153BD1CA-CFD0-4112-B0C0-0B1B9E57E002}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5035,7 +5035,7 @@
           </x14:formula2>
           <xm:sqref>M18</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{5BA9EDB5-FAA8-442E-A272-829D481337B1}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{10040218-07D9-4C18-A47C-51986CB9FD68}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5044,7 +5044,7 @@
           </x14:formula2>
           <xm:sqref>M19</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0D161274-75A8-4376-A47B-6231B5293CDC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{391196E1-7DD8-42D8-B7E3-A7F2A5781A84}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5053,7 +5053,7 @@
           </x14:formula2>
           <xm:sqref>M20</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{26EF87F1-9D25-4E71-99D3-C228C0AD0ABA}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{24D52F3B-93E5-4154-A04D-A55F6843B748}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5062,7 +5062,7 @@
           </x14:formula2>
           <xm:sqref>M21</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{46B6FE8D-85BF-4C62-A2BB-31E5587AF890}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{412ADD45-4CCF-4022-B95D-4C73F5B82CF2}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5071,7 +5071,7 @@
           </x14:formula2>
           <xm:sqref>M23</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{4F431A2B-2B6C-4F38-BDA1-E79BD29CC40E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{65667420-CC0D-4FCA-B6F9-F172EB96EA05}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5080,7 +5080,7 @@
           </x14:formula2>
           <xm:sqref>M24</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{4D05FD78-F0B5-4334-8BE9-89F61249A41C}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{3D30BD1A-BF25-4BEA-8E6F-728FCEDAD285}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5089,7 +5089,7 @@
           </x14:formula2>
           <xm:sqref>M25</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{7C9A1D03-7531-49DB-8965-ED0D4A458743}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{58F08322-8017-4C55-B344-74A1B86959E4}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
@@ -5212,7 +5212,7 @@
         <v>195</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N2" s="15"/>
       <c r="O2" s="15"/>
@@ -5255,7 +5255,7 @@
         <v>195</v>
       </c>
       <c r="M3" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N3" s="15"/>
       <c r="O3" s="15"/>
@@ -5298,7 +5298,7 @@
         <v>195</v>
       </c>
       <c r="M4" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N4" s="15"/>
       <c r="O4" s="15"/>
@@ -5341,7 +5341,7 @@
         <v>195</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N5" s="15"/>
       <c r="O5" s="15" t="s">
@@ -5386,7 +5386,7 @@
         <v>219</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
@@ -5429,7 +5429,7 @@
         <v>219</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N7" s="15"/>
       <c r="O7" s="15"/>
@@ -5472,7 +5472,7 @@
         <v>230</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
@@ -5515,7 +5515,7 @@
         <v>230</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N9" s="15"/>
       <c r="O9" s="15"/>
@@ -5558,7 +5558,7 @@
         <v>242</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N10" s="15"/>
       <c r="O10" s="15"/>
@@ -5601,7 +5601,7 @@
         <v>242</v>
       </c>
       <c r="M11" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N11" s="15"/>
       <c r="O11" s="15"/>
@@ -5644,7 +5644,7 @@
         <v>242</v>
       </c>
       <c r="M12" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N12" s="15"/>
       <c r="O12" s="15"/>
@@ -5687,7 +5687,7 @@
         <v>259</v>
       </c>
       <c r="M13" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N13" s="15"/>
       <c r="O13" s="15"/>
@@ -5730,7 +5730,7 @@
         <v>266</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N14" s="15"/>
       <c r="O14" s="15"/>
@@ -5773,7 +5773,7 @@
         <v>266</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N15" s="15"/>
       <c r="O15" s="15"/>
@@ -5816,7 +5816,7 @@
         <v>195</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="15" t="s">
@@ -5861,7 +5861,7 @@
         <v>219</v>
       </c>
       <c r="M17" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N17" s="15"/>
       <c r="O17" s="15"/>
@@ -5904,7 +5904,7 @@
         <v>195</v>
       </c>
       <c r="M18" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N18" s="15"/>
       <c r="O18" s="15"/>
@@ -5947,7 +5947,7 @@
         <v>266</v>
       </c>
       <c r="M19" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N19" s="15"/>
       <c r="O19" s="15"/>
@@ -6017,15 +6017,153 @@
           </x14:cfRule>
           <xm:sqref>M2:M19</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M15:M16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M15:M16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M15:M16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>M17:M19</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{249AFDEA-C53C-44E5-B19A-4A3831F35E64}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3" disablePrompts="0">
+        <x14:dataValidation xr:uid="{523F2BC9-A78A-4AF6-95EB-35D661DC0BF7}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>
-          <xm:sqref>M2:M19</xm:sqref>
+          <xm:sqref>M2:M14</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{41A20C3C-8B84-4CF1-9E96-9528D1DC79EF}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <xm:sqref>M15:M16</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{668078D8-A191-41E2-B1B4-75B364D4C617}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <xm:sqref>M17:M19</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -6784,7 +6922,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{3E07C439-6CF5-429E-A749-7899EFA7F43D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{1BA9D181-C2EF-4231-9122-93ACF90C89AB}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
           </x14:formula1>

</xml_diff>